<commit_message>
doc(doc): Modification du jdt
</commit_message>
<xml_diff>
--- a/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
+++ b/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi41dcg\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi41dcg\Documents\GitHub\ReadMe\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B48EBF-7ED6-4111-9085-2EC2797607F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05DF8AE-CB01-46E6-A2ED-F9D40D15A83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -145,6 +145,12 @@
   </si>
   <si>
     <t>Affichage des livres de la db et rédirection sur la page de cette livre si je clique</t>
+  </si>
+  <si>
+    <t>Migration de la base locale à API pout fetcher les livres</t>
+  </si>
+  <si>
+    <t>Les données ne voulaient pas s'afficher</t>
   </si>
 </sst>
 </file>
@@ -1049,7 +1055,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.20833333333333334</c:v>
+                  <c:v>0.28472222222222221</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2027,7 +2033,7 @@
       </c>
       <c r="C3" s="24" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 7 heurs 30 minutes</v>
+        <v>0 jours 9 heurs 20 minutes</v>
       </c>
       <c r="D3" s="24"/>
       <c r="E3" s="3"/>
@@ -2042,15 +2048,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="24">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>360</v>
+        <v>420</v>
       </c>
       <c r="D4" s="24">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="E4" s="51">
         <f>SUM(C4:D4)</f>
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2199,13 +2205,27 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="19"/>
+      <c r="A11" s="17">
+        <v>17</v>
+      </c>
+      <c r="B11" s="39">
+        <v>46134</v>
+      </c>
+      <c r="C11" s="35">
+        <v>1</v>
+      </c>
+      <c r="D11" s="43">
+        <v>50</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>36</v>
+      </c>
       <c r="M11" t="s">
         <v>6</v>
       </c>
@@ -8202,11 +8222,11 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="C5" s="52" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8214,7 +8234,7 @@
       </c>
       <c r="D5" s="44">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.20833333333333334</v>
+        <v>0.28472222222222221</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8323,7 +8343,7 @@
       </c>
       <c r="D12" s="45">
         <f>SUM(D4:D11)</f>
-        <v>0.22916666666666669</v>
+        <v>0.30555555555555552</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8345,6 +8365,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD12CA962D3BC343BA4881942FCA9ABD" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="69c7e1234aa399a5294368cedfc9727e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb2b4dc0-5538-4988-a426-1e3bf3687743" xmlns:ns3="26488081-7094-48e3-a435-bbb366c5709a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f55906f2b711226ab16b0d1a2f445893" ns2:_="" ns3:_="">
     <xsd:import namespace="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
@@ -8551,17 +8582,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -8571,6 +8591,19 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
+    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8587,17 +8620,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
-    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
doc(jdt): mise à jour du JdT
</commit_message>
<xml_diff>
--- a/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
+++ b/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi41dcg\Documents\GitHub\ReadMe\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52AD68E6-AAB7-4C55-A14F-05CB688A4E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAAD1D62-B502-4DD4-9840-785837151F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -151,6 +151,15 @@
   </si>
   <si>
     <t>Les données ne voulaient pas s'afficher</t>
+  </si>
+  <si>
+    <t>Affichage des epubs des livres : appel des fichiers du dossier pendant clique sur le livre et ouverture dans WebView</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sauvegarde du progres et récupération lors prochain ouverture </t>
+  </si>
+  <si>
+    <t>Améliorations du design de l'application</t>
   </si>
 </sst>
 </file>
@@ -1055,7 +1064,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.28472222222222221</c:v>
+                  <c:v>0.35069444444444442</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1070,7 +1079,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.0833333333333332E-2</c:v>
+                  <c:v>5.5555555555555552E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -2033,7 +2042,7 @@
       </c>
       <c r="C3" s="24" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 9 heurs 20 minutes</v>
+        <v>0 jours 11 heurs 45 minutes</v>
       </c>
       <c r="D3" s="24"/>
       <c r="E3" s="3"/>
@@ -2052,11 +2061,11 @@
       </c>
       <c r="D4" s="24">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>140</v>
+        <v>285</v>
       </c>
       <c r="E4" s="51">
         <f>SUM(C4:D4)</f>
-        <v>560</v>
+        <v>705</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2236,11 +2245,20 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="38"/>
+    <row r="12" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B12" s="38">
+        <v>46141</v>
+      </c>
       <c r="C12" s="34"/>
-      <c r="D12" s="42"/>
-      <c r="F12" s="47"/>
+      <c r="D12" s="42">
+        <v>45</v>
+      </c>
+      <c r="E12" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="47" t="s">
+        <v>37</v>
+      </c>
       <c r="G12" s="16"/>
       <c r="M12" t="s">
         <v>7</v>
@@ -2254,11 +2272,19 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
-      <c r="B13" s="39"/>
+      <c r="B13" s="39">
+        <v>46141</v>
+      </c>
       <c r="C13" s="35"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="47"/>
+      <c r="D13" s="43">
+        <v>50</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="47" t="s">
+        <v>38</v>
+      </c>
       <c r="G13" s="19"/>
       <c r="M13" t="s">
         <v>8</v>
@@ -2271,10 +2297,19 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="38"/>
+      <c r="B14" s="38">
+        <v>46141</v>
+      </c>
       <c r="C14" s="34"/>
-      <c r="D14" s="42"/>
-      <c r="F14" s="47"/>
+      <c r="D14" s="42">
+        <v>50</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="47" t="s">
+        <v>39</v>
+      </c>
       <c r="G14" s="16"/>
       <c r="M14" t="s">
         <v>24</v>
@@ -8226,7 +8261,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>110</v>
+        <v>205</v>
       </c>
       <c r="C5" s="52" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8234,7 +8269,7 @@
       </c>
       <c r="D5" s="44">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.28472222222222221</v>
+        <v>0.35069444444444442</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8312,7 +8347,7 @@
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C10,'Journal de travail'!$D$7:$D$532)</f>
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="C10" s="48" t="str">
         <f>'Journal de travail'!M14</f>
@@ -8320,7 +8355,7 @@
       </c>
       <c r="D10" s="44">
         <f t="shared" si="0"/>
-        <v>2.0833333333333332E-2</v>
+        <v>5.5555555555555552E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -8343,7 +8378,7 @@
       </c>
       <c r="D12" s="45">
         <f>SUM(D4:D11)</f>
-        <v>0.30555555555555552</v>
+        <v>0.40625</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8356,26 +8391,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD12CA962D3BC343BA4881942FCA9ABD" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="69c7e1234aa399a5294368cedfc9727e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb2b4dc0-5538-4988-a426-1e3bf3687743" xmlns:ns3="26488081-7094-48e3-a435-bbb366c5709a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f55906f2b711226ab16b0d1a2f445893" ns2:_="" ns3:_="">
     <xsd:import namespace="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
@@ -8582,10 +8597,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
+    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8604,20 +8650,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
-    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(app): ajout de l'ajout des livres
</commit_message>
<xml_diff>
--- a/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
+++ b/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi41dcg\Documents\GitHub\ReadMe\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAAD1D62-B502-4DD4-9840-785837151F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A18B5F-9769-4823-8680-010D34EA3DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -160,6 +160,15 @@
   </si>
   <si>
     <t>Améliorations du design de l'application</t>
+  </si>
+  <si>
+    <t>Ajout des tags pour les livres, pour le moment seulement l'apparence</t>
+  </si>
+  <si>
+    <t>Ajout des livres dans app via formulaire</t>
+  </si>
+  <si>
+    <t>ça cassait le titre du livre</t>
   </si>
 </sst>
 </file>
@@ -793,7 +802,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1064,7 +1073,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.35069444444444442</c:v>
+                  <c:v>0.41666666666666669</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2042,7 +2051,7 @@
       </c>
       <c r="C3" s="24" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 11 heurs 45 minutes</v>
+        <v>0 jours 13 heurs 20 minutes</v>
       </c>
       <c r="D3" s="24"/>
       <c r="E3" s="3"/>
@@ -2057,15 +2066,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="24">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="D4" s="24">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>285</v>
+        <v>320</v>
       </c>
       <c r="E4" s="51">
         <f>SUM(C4:D4)</f>
-        <v>705</v>
+        <v>800</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2323,11 +2332,19 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="17"/>
-      <c r="B15" s="39"/>
+      <c r="B15" s="39">
+        <v>46148</v>
+      </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="47"/>
+      <c r="D15" s="43">
+        <v>35</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="47" t="s">
+        <v>40</v>
+      </c>
       <c r="G15" s="19"/>
       <c r="M15" t="s">
         <v>25</v>
@@ -2340,11 +2357,22 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="38"/>
-      <c r="C16" s="34"/>
+      <c r="B16" s="38">
+        <v>46148</v>
+      </c>
+      <c r="C16" s="34">
+        <v>1</v>
+      </c>
       <c r="D16" s="42"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="16"/>
+      <c r="E16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>42</v>
+      </c>
       <c r="O16">
         <v>40</v>
       </c>
@@ -8257,11 +8285,11 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="C5" s="52" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8269,7 +8297,7 @@
       </c>
       <c r="D5" s="44">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.35069444444444442</v>
+        <v>0.41666666666666669</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8378,7 +8406,7 @@
       </c>
       <c r="D12" s="45">
         <f>SUM(D4:D11)</f>
-        <v>0.40625</v>
+        <v>0.47222222222222221</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8391,6 +8419,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD12CA962D3BC343BA4881942FCA9ABD" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="69c7e1234aa399a5294368cedfc9727e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb2b4dc0-5538-4988-a426-1e3bf3687743" xmlns:ns3="26488081-7094-48e3-a435-bbb366c5709a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f55906f2b711226ab16b0d1a2f445893" ns2:_="" ns3:_="">
     <xsd:import namespace="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
@@ -8597,41 +8645,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
-    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8650,9 +8667,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
+    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(book) fixe du mone du livre qui s'efface
</commit_message>
<xml_diff>
--- a/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
+++ b/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi41dcg\Documents\GitHub\ReadMe\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A18B5F-9769-4823-8680-010D34EA3DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEE3A312-73AA-4DF9-B6FC-628BE36454E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -169,6 +169,18 @@
   </si>
   <si>
     <t>ça cassait le titre du livre</t>
+  </si>
+  <si>
+    <t>Règlage du problème avec les titres [WiP]</t>
+  </si>
+  <si>
+    <t>Règlage du problème avec les titres [DONE]</t>
+  </si>
+  <si>
+    <t>Ajout de la suppression des livres</t>
+  </si>
+  <si>
+    <t>Ajout des tags fonctionnels pour les livres</t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1085,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.41666666666666669</c:v>
+                  <c:v>0.53472222222222221</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2051,7 +2063,7 @@
       </c>
       <c r="C3" s="24" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 13 heurs 20 minutes</v>
+        <v>0 jours 16 heurs 10 minutes</v>
       </c>
       <c r="D3" s="24"/>
       <c r="E3" s="3"/>
@@ -2070,11 +2082,11 @@
       </c>
       <c r="D4" s="24">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>320</v>
+        <v>490</v>
       </c>
       <c r="E4" s="51">
         <f>SUM(C4:D4)</f>
-        <v>800</v>
+        <v>970</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2379,21 +2391,38 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="17"/>
-      <c r="B17" s="39"/>
+      <c r="B17" s="39">
+        <v>46148</v>
+      </c>
       <c r="C17" s="35"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="47"/>
+      <c r="D17" s="43">
+        <v>45</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>43</v>
+      </c>
       <c r="G17" s="19"/>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="38"/>
+      <c r="B18" s="38">
+        <v>46155</v>
+      </c>
       <c r="C18" s="34"/>
-      <c r="D18" s="42"/>
-      <c r="F18" s="47"/>
+      <c r="D18" s="42">
+        <v>45</v>
+      </c>
+      <c r="E18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18" s="47" t="s">
+        <v>44</v>
+      </c>
       <c r="G18" s="16"/>
       <c r="O18">
         <v>50</v>
@@ -2401,21 +2430,38 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="17"/>
-      <c r="B19" s="39"/>
+      <c r="B19" s="39">
+        <v>46155</v>
+      </c>
       <c r="C19" s="35"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="47"/>
+      <c r="D19" s="43">
+        <v>45</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19" s="47" t="s">
+        <v>45</v>
+      </c>
       <c r="G19" s="19"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B20" s="38"/>
+      <c r="B20" s="38">
+        <v>46155</v>
+      </c>
       <c r="C20" s="34"/>
-      <c r="D20" s="42"/>
-      <c r="F20" s="47"/>
+      <c r="D20" s="42">
+        <v>35</v>
+      </c>
+      <c r="E20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F20" s="47" t="s">
+        <v>46</v>
+      </c>
       <c r="G20" s="16"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -8289,7 +8335,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>240</v>
+        <v>410</v>
       </c>
       <c r="C5" s="52" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8297,7 +8343,7 @@
       </c>
       <c r="D5" s="44">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.41666666666666669</v>
+        <v>0.53472222222222221</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8406,7 +8452,7 @@
       </c>
       <c r="D12" s="45">
         <f>SUM(D4:D11)</f>
-        <v>0.47222222222222221</v>
+        <v>0.59027777777777779</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8419,26 +8465,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD12CA962D3BC343BA4881942FCA9ABD" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="69c7e1234aa399a5294368cedfc9727e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb2b4dc0-5538-4988-a426-1e3bf3687743" xmlns:ns3="26488081-7094-48e3-a435-bbb366c5709a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f55906f2b711226ab16b0d1a2f445893" ns2:_="" ns3:_="">
     <xsd:import namespace="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
@@ -8645,10 +8671,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
+    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8667,20 +8724,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
-    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(tags)ajout de l'ajout des tags pour les livres
</commit_message>
<xml_diff>
--- a/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
+++ b/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi41dcg\Documents\GitHub\ReadMe\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEE3A312-73AA-4DF9-B6FC-628BE36454E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F6CA9C-2CFF-4E0B-AF1A-127D0CBDE7F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="48">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>Ajout des tags fonctionnels pour les livres</t>
+  </si>
+  <si>
+    <t>Ajout de l'ajout des tags</t>
   </si>
 </sst>
 </file>
@@ -1085,7 +1088,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.53472222222222221</c:v>
+                  <c:v>0.55555555555555558</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2063,7 +2066,7 @@
       </c>
       <c r="C3" s="24" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 16 heurs 10 minutes</v>
+        <v>0 jours 16 heurs 39 minutes</v>
       </c>
       <c r="D3" s="24"/>
       <c r="E3" s="3"/>
@@ -2082,11 +2085,11 @@
       </c>
       <c r="D4" s="24">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>490</v>
+        <v>520</v>
       </c>
       <c r="E4" s="51">
         <f>SUM(C4:D4)</f>
-        <v>970</v>
+        <v>1000</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2466,11 +2469,19 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
-      <c r="B21" s="39"/>
+      <c r="B21" s="39">
+        <v>46162</v>
+      </c>
       <c r="C21" s="35"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="47"/>
+      <c r="D21" s="43">
+        <v>30</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="47" t="s">
+        <v>47</v>
+      </c>
       <c r="G21" s="19"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -8335,7 +8346,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>410</v>
+        <v>440</v>
       </c>
       <c r="C5" s="52" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8343,7 +8354,7 @@
       </c>
       <c r="D5" s="44">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.53472222222222221</v>
+        <v>0.55555555555555558</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8452,7 +8463,7 @@
       </c>
       <c r="D12" s="45">
         <f>SUM(D4:D11)</f>
-        <v>0.59027777777777779</v>
+        <v>0.61111111111111116</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8465,6 +8476,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD12CA962D3BC343BA4881942FCA9ABD" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="69c7e1234aa399a5294368cedfc9727e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb2b4dc0-5538-4988-a426-1e3bf3687743" xmlns:ns3="26488081-7094-48e3-a435-bbb366c5709a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f55906f2b711226ab16b0d1a2f445893" ns2:_="" ns3:_="">
     <xsd:import namespace="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
@@ -8671,41 +8702,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
-    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8724,9 +8724,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
+    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(app): Retouches finales sur le projet
</commit_message>
<xml_diff>
--- a/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
+++ b/doc/Journal-de-Travail_BorodkinOlkesandrStepanovych.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi41dcg\Documents\GitHub\ReadMe\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F6CA9C-2CFF-4E0B-AF1A-127D0CBDE7F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA113F8-8C16-4CFF-AC7A-89EA49115E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="50">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -184,6 +184,12 @@
   </si>
   <si>
     <t>Ajout de l'ajout des tags</t>
+  </si>
+  <si>
+    <t>Ajout des scénarios du test pour l'application</t>
+  </si>
+  <si>
+    <t>Les retouches finales sur le projet</t>
   </si>
 </sst>
 </file>
@@ -1088,10 +1094,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.55555555555555558</c:v>
+                  <c:v>0.59722222222222221</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>2.0833333333333332E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2066,7 +2072,7 @@
       </c>
       <c r="C3" s="24" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 16 heurs 39 minutes</v>
+        <v>0 jours 18 heurs 9 minutes</v>
       </c>
       <c r="D3" s="24"/>
       <c r="E3" s="3"/>
@@ -2081,15 +2087,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="24">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>480</v>
+        <v>540</v>
       </c>
       <c r="D4" s="24">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="E4" s="51">
         <f>SUM(C4:D4)</f>
-        <v>1000</v>
+        <v>1090</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2485,19 +2491,36 @@
       <c r="G21" s="19"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="38"/>
+      <c r="B22" s="38">
+        <v>46162</v>
+      </c>
       <c r="C22" s="34"/>
-      <c r="D22" s="42"/>
-      <c r="F22" s="47"/>
+      <c r="D22" s="42">
+        <v>30</v>
+      </c>
+      <c r="E22" t="s">
+        <v>5</v>
+      </c>
+      <c r="F22" s="47" t="s">
+        <v>48</v>
+      </c>
       <c r="G22" s="16"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
-      <c r="B23" s="39"/>
-      <c r="C23" s="35"/>
+      <c r="B23" s="39">
+        <v>46162</v>
+      </c>
+      <c r="C23" s="35">
+        <v>1</v>
+      </c>
       <c r="D23" s="43"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="47"/>
+      <c r="E23" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" s="47" t="s">
+        <v>49</v>
+      </c>
       <c r="G23" s="19"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -8342,7 +8365,7 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>360</v>
+        <v>420</v>
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
@@ -8354,7 +8377,7 @@
       </c>
       <c r="D5" s="44">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.55555555555555558</v>
+        <v>0.59722222222222221</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8364,7 +8387,7 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C6" s="28" t="str">
         <f>'Journal de travail'!M10</f>
@@ -8372,7 +8395,7 @@
       </c>
       <c r="D6" s="44">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.0833333333333332E-2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -8463,7 +8486,7 @@
       </c>
       <c r="D12" s="45">
         <f>SUM(D4:D11)</f>
-        <v>0.61111111111111116</v>
+        <v>0.67361111111111116</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8476,26 +8499,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD12CA962D3BC343BA4881942FCA9ABD" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="69c7e1234aa399a5294368cedfc9727e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb2b4dc0-5538-4988-a426-1e3bf3687743" xmlns:ns3="26488081-7094-48e3-a435-bbb366c5709a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f55906f2b711226ab16b0d1a2f445893" ns2:_="" ns3:_="">
     <xsd:import namespace="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
@@ -8702,10 +8705,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
+    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8724,20 +8758,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB911C2A-3E3E-4AFD-88DE-B1DD58AC65DD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
-    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>